<commit_message>
Add Mutual DX and suffix-safe matching
This release adds suffix-safe patient matching across the schedule and Mutual workbook, so names like `Marchetti Jr` match their plain remit form without rewriting stored names. Newly appended names are now title-cased to match the sheet’s style, while existing rows remain untouched.

It also adds the optional `List_of_Patients_Mutual.xlsx` DX lookup, fills blank DX values on rows the app is already touching, flags conflicts and low-confidence matches for review, and stamps `Processed On` / `Remit Check/EFT #` audit columns on touched rows. The change keeps the existing safety guarantees intact: never overwrite, dedupe/idempotency, preview-confirm-download flow, and whole-workbook preservation.
</commit_message>
<xml_diff>
--- a/tests/fixtures/List_of_Patients_Schedule.xlsx
+++ b/tests/fixtures/List_of_Patients_Schedule.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -835,7 +835,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Delacroix, Owen</t>
+          <t>Bystritskaya Jr, Anna</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -844,7 +844,7 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>46027</v>
+        <v>46126</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -853,12 +853,39 @@
       </c>
       <c r="E12" s="4" t="n"/>
       <c r="F12" s="4" t="n"/>
-      <c r="J12" t="inlineStr">
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>99213/90833</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Delacroix, Owen</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Medicare</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>46027</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2/32/26</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="n"/>
+      <c r="F13" s="4" t="n"/>
+      <c r="J13" t="inlineStr">
         <is>
           <t>F41.1, F32.9</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>99213/90833</t>
         </is>

</xml_diff>